<commit_message>
Embed witan-rendered result charts in README
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/charts/charts.xlsx
+++ b/charts/charts.xlsx
@@ -129,8 +129,8 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>FUSE — 10,544 wild-web workbooks
-xlsx engines — top-right is best</a:t>
+              <a:t>xlsx engines — top-right is best
+FUSE — 10,544 wild-web workbooks</a:t>
             </a:r>
             <a:endParaRPr/>
           </a:p>
@@ -786,8 +786,8 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>SpreadsheetBench — 5,426 forum workbooks
-xlsx engines — top-right is best</a:t>
+              <a:t>xlsx engines — top-right is best
+SpreadsheetBench — 5,426 forum workbooks</a:t>
             </a:r>
             <a:endParaRPr/>
           </a:p>

</xml_diff>

<commit_message>
Charts: unlabeled headroom sliver so the 100% boundary marker renders whole
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/charts/charts.xlsx
+++ b/charts/charts.xlsx
@@ -435,7 +435,7 @@
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0.94"/>
-          <c:max val="1"/>
+          <c:max val="1.005"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
@@ -1092,7 +1092,7 @@
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0.96"/>
-          <c:max val="1"/>
+          <c:max val="1.005"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>

</xml_diff>